<commit_message>
Rating update + 2 new tourney evaluations
Почався новий сезон -- 25/26. Внесено  турніри Чумацький Шлях 2, СинЛУК Зима
</commit_message>
<xml_diff>
--- a/output/pl1takdl.xlsx
+++ b/output/pl1takdl.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Назва</t>
   </si>
@@ -95,6 +95,12 @@
   </si>
   <si>
     <t>Борисфен 12: Верхня Хортиця</t>
+  </si>
+  <si>
+    <t>Поки зорить Чумацький Шлях 2</t>
+  </si>
+  <si>
+    <t>Синхрон ЛУК 25/26. Зима</t>
   </si>
 </sst>
 </file>
@@ -452,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -663,6 +669,22 @@
         <v>3.46</v>
       </c>
     </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27">
+        <v>4.14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28">
+        <v>3.81</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>